<commit_message>
se corrigio los xlsx de ejemplo
</commit_message>
<xml_diff>
--- a/temp/asignaturas_2025-11-18.xlsx
+++ b/temp/asignaturas_2025-11-18.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\BD3\Project\Proyecto-DB3\temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68B0574C-1008-4176-B0D6-3399BB2AD4C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9E23797-EEDE-4AD9-911E-2A321AFA06E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28690" yWindow="-110" windowWidth="29020" windowHeight="15700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,18 +46,12 @@
     <t>Materia separada</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>Castellano y Literatura</t>
   </si>
   <si>
     <t>Alta carga troncal</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>Castellano y Literatura (Técnico)</t>
   </si>
   <si>
@@ -143,6 +137,12 @@
   </si>
   <si>
     <t>Horas Semanales</t>
+  </si>
+  <si>
+    <t>Aula Genérica</t>
+  </si>
+  <si>
+    <t>Espacio Especializado</t>
   </si>
 </sst>
 </file>
@@ -517,6 +517,9 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="24.6640625" customWidth="1"/>
+    <col min="4" max="4" width="23.25" customWidth="1"/>
+    <col min="5" max="5" width="26.25" customWidth="1"/>
+    <col min="6" max="6" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -524,7 +527,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -559,7 +562,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G2">
         <v>3</v>
@@ -567,13 +570,13 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -582,7 +585,7 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -590,13 +593,13 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4">
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -605,7 +608,7 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G4">
         <v>2</v>
@@ -613,13 +616,13 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5">
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -628,7 +631,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G5">
         <v>3</v>
@@ -636,13 +639,13 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B6">
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -651,7 +654,7 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G6">
         <v>4</v>
@@ -659,13 +662,13 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B7">
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -674,7 +677,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G7">
         <v>5</v>
@@ -682,13 +685,13 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B8">
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -697,7 +700,7 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G8">
         <v>1</v>
@@ -705,13 +708,13 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B9">
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -720,7 +723,7 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G9">
         <v>2</v>
@@ -728,13 +731,13 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B10">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -743,7 +746,7 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G10">
         <v>5</v>
@@ -751,13 +754,13 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B11">
         <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -766,7 +769,7 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G11">
         <v>1</v>
@@ -774,13 +777,13 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B12">
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -789,7 +792,7 @@
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G12">
         <v>2</v>
@@ -797,13 +800,13 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -812,7 +815,7 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G13">
         <v>3</v>
@@ -820,13 +823,13 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B14">
         <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -835,7 +838,7 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G14">
         <v>4</v>
@@ -843,13 +846,13 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B15">
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -858,7 +861,7 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G15">
         <v>5</v>
@@ -866,13 +869,13 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B16">
         <v>4</v>
       </c>
       <c r="C16" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D16">
         <v>2</v>
@@ -881,7 +884,7 @@
         <v>4</v>
       </c>
       <c r="F16" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -889,13 +892,13 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B17">
         <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D17">
         <v>2</v>
@@ -904,7 +907,7 @@
         <v>4</v>
       </c>
       <c r="F17" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G17">
         <v>2</v>
@@ -912,13 +915,13 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B18">
         <v>4</v>
       </c>
       <c r="C18" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D18">
         <v>2</v>
@@ -927,7 +930,7 @@
         <v>4</v>
       </c>
       <c r="F18" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G18">
         <v>3</v>
@@ -935,13 +938,13 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -950,7 +953,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -958,13 +961,13 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B20">
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -973,7 +976,7 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G20">
         <v>2</v>
@@ -981,13 +984,13 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -996,7 +999,7 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G21">
         <v>3</v>
@@ -1004,7 +1007,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B22">
         <v>4</v>
@@ -1019,7 +1022,7 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G22">
         <v>3</v>
@@ -1027,13 +1030,13 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B23">
         <v>4</v>
       </c>
       <c r="C23" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -1042,7 +1045,7 @@
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G23">
         <v>4</v>
@@ -1050,13 +1053,13 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B24">
         <v>3</v>
       </c>
       <c r="C24" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -1065,7 +1068,7 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G24">
         <v>5</v>
@@ -1073,13 +1076,13 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B25">
         <v>3</v>
       </c>
       <c r="C25" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -1088,7 +1091,7 @@
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G25">
         <v>4</v>
@@ -1096,13 +1099,13 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B26">
         <v>3</v>
       </c>
       <c r="C26" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -1111,7 +1114,7 @@
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G26">
         <v>1</v>
@@ -1119,13 +1122,13 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B27">
         <v>3</v>
       </c>
       <c r="C27" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -1134,7 +1137,7 @@
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G27">
         <v>2</v>
@@ -1142,13 +1145,13 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B28">
         <v>3</v>
       </c>
       <c r="C28" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -1157,7 +1160,7 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G28">
         <v>3</v>
@@ -1165,13 +1168,13 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B29">
         <v>3</v>
       </c>
       <c r="C29" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -1180,7 +1183,7 @@
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G29">
         <v>4</v>
@@ -1188,13 +1191,13 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B30">
         <v>3</v>
       </c>
       <c r="C30" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -1203,7 +1206,7 @@
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G30">
         <v>5</v>
@@ -1211,13 +1214,13 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B31">
         <v>2</v>
       </c>
       <c r="C31" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D31">
         <v>1</v>
@@ -1226,7 +1229,7 @@
         <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G31">
         <v>4</v>
@@ -1234,13 +1237,13 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B32">
         <v>2</v>
       </c>
       <c r="C32" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D32">
         <v>1</v>
@@ -1249,7 +1252,7 @@
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G32">
         <v>5</v>
@@ -1257,13 +1260,13 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B33">
         <v>5</v>
       </c>
       <c r="C33" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D33">
         <v>1</v>
@@ -1272,7 +1275,7 @@
         <v>1</v>
       </c>
       <c r="F33" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G33">
         <v>1</v>
@@ -1280,13 +1283,13 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B34">
         <v>5</v>
       </c>
       <c r="C34" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D34">
         <v>1</v>
@@ -1295,7 +1298,7 @@
         <v>1</v>
       </c>
       <c r="F34" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G34">
         <v>2</v>
@@ -1303,13 +1306,13 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B35">
         <v>5</v>
       </c>
       <c r="C35" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D35">
         <v>1</v>
@@ -1318,7 +1321,7 @@
         <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G35">
         <v>3</v>
@@ -1326,13 +1329,13 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B36">
         <v>4</v>
       </c>
       <c r="C36" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D36">
         <v>1</v>
@@ -1341,7 +1344,7 @@
         <v>1</v>
       </c>
       <c r="F36" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G36">
         <v>4</v>
@@ -1349,13 +1352,13 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B37">
         <v>4</v>
       </c>
       <c r="C37" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D37">
         <v>1</v>
@@ -1364,7 +1367,7 @@
         <v>1</v>
       </c>
       <c r="F37" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G37">
         <v>5</v>
@@ -1372,13 +1375,13 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B38">
         <v>10</v>
       </c>
       <c r="C38" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D38">
         <v>2</v>
@@ -1387,7 +1390,7 @@
         <v>3</v>
       </c>
       <c r="F38" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G38">
         <v>4</v>
@@ -1395,13 +1398,13 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B39">
         <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D39">
         <v>2</v>
@@ -1410,7 +1413,7 @@
         <v>3</v>
       </c>
       <c r="F39" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G39">
         <v>5</v>
@@ -1418,7 +1421,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B40">
         <v>4</v>
@@ -1433,7 +1436,7 @@
         <v>1</v>
       </c>
       <c r="F40" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G40">
         <v>3</v>
@@ -1441,13 +1444,13 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B41">
         <v>4</v>
       </c>
       <c r="C41" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -1456,7 +1459,7 @@
         <v>1</v>
       </c>
       <c r="F41" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G41">
         <v>4</v>
@@ -1464,13 +1467,13 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B42">
         <v>2</v>
       </c>
       <c r="C42" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D42">
         <v>1</v>
@@ -1479,7 +1482,7 @@
         <v>1</v>
       </c>
       <c r="F42" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G42">
         <v>4</v>
@@ -1487,13 +1490,13 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B43">
         <v>2</v>
       </c>
       <c r="C43" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D43">
         <v>1</v>
@@ -1502,7 +1505,7 @@
         <v>1</v>
       </c>
       <c r="F43" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="G43">
         <v>5</v>
@@ -1510,5 +1513,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>